<commit_message>
Fix Colour x Size bulk upload: parent SKU grouping, sizes and error reporting.
A repeated Parent SKU is how the sheet groups colours, but the wizard read it as the variant SKU and rejected the file for duplicate SKUs. Parent, Variant and Image SKU columns are now kept apart, uniqueness applies to the variant SKU only, and a colour row may list its sizes together. Errors name the variant SKU instead of the parent, the completion screen no longer reports success when nothing was accepted, and Single Listing keeps one colour.
</commit_message>
<xml_diff>
--- a/public/bulk-listing-templates/IERADA_Bulk_Listing_Color_Size_Variations.xlsx
+++ b/public/bulk-listing-templates/IERADA_Bulk_Listing_Color_Size_Variations.xlsx
@@ -24,7 +24,7 @@
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>Admin Size attributes. One size per variation row.</t>
+          <t>One colour per row. Sizes can be comma-separated. Parent SKU repeats; Variant SKU is unique per colour.</t>
         </r>
       </text>
     </comment>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="253">
   <si>
     <t>IERADA Seller Panel</t>
   </si>
@@ -104,16 +104,34 @@
     <t>What you fill vs what AI fills</t>
   </si>
   <si>
-    <t>Products sheet: fill parent SKU, brand, package, and What's in the Box yourself. Variations sheet: colour, size, variant SKU, Image SKU, price, stock. Template columns are never written by AI.</t>
+    <t>Products sheet: one parent SKU per listing, plus brand, package, and What's in the Box. Do not put colour or size on the Products sheet.</t>
+  </si>
+  <si>
+    <t>Variations sheet: one row per colour under the same parent SKU. Each colour needs a unique Variant SKU. Size can be one value, or several on that colour row (6,7,8,9).</t>
   </si>
   <si>
     <t>AI fills parent copy (description, features, SEO) after validate. On Step 4 download the completed workbook, edit, and re-upload on Preview — then submit.</t>
   </si>
   <si>
+    <t>How Colour × Size variations work</t>
+  </si>
+  <si>
+    <t>Same parent SKU on every variation row groups them into one listing. Repeating the parent SKU is required — it is not a duplicate SKU.</t>
+  </si>
+  <si>
+    <t>One colour per Variations row. You may list sizes as 6,7,8,9 on that row (we create one size variation each and append the size to the Variant SKU) or use one size per row with its own Variant SKU.</t>
+  </si>
+  <si>
+    <t>Variant SKU must be unique per colour (lifeo-zimmi-brown-277). Image SKU can stay at colour level so all sizes of Brown share the same photos.</t>
+  </si>
+  <si>
     <t>Size dropdown (admin Size attributes)</t>
   </si>
   <si>
-    <t>Variations → Size is a dropdown of live admin Size attributes. Pick one size per variation row.</t>
+    <t>Variations → Size is a dropdown of live admin Size attributes. One size per row, or several sizes on one colour row separated by commas.</t>
+  </si>
+  <si>
+    <t>Kids Fashion: choose an age-group size so buyers understand the fit — 6-9 Months, 9-12 Months, 12-15 Months, 18-21 Months, 2-2.5 Years, 3-3.5 Years, 5-5.5 Years. Do not use adult S/M/L for kids apparel.</t>
   </si>
   <si>
     <t>Image SKU (recommended)</t>
@@ -206,7 +224,7 @@
     <t>colour</t>
   </si>
   <si>
-    <t>Catalogue colour. Images are shared at colour level.</t>
+    <t>One catalogue colour for this variation row. Add another row for a second colour under the same parent SKU.</t>
   </si>
   <si>
     <t>Size</t>
@@ -215,7 +233,7 @@
     <t>size</t>
   </si>
   <si>
-    <t>Pick one catalogue size from the dropdown (admin Size attributes).</t>
+    <t>One size, or several on this colour row as 6,7,8,9. Kids Fashion: pick age-group sizes (6-9 Months, 2-2.5 Years).</t>
   </si>
   <si>
     <t>Variant SKU</t>
@@ -224,7 +242,7 @@
     <t>variant_sku</t>
   </si>
   <si>
-    <t>Unique SKU for this colour × size row.</t>
+    <t>Unique SKU for this colour. Repeating the Parent SKU is required and is not a duplicate.</t>
   </si>
   <si>
     <t>Image SKU</t>
@@ -506,70 +524,193 @@
     <t>• Prefer Image SKU at colour level. Example files: FAS-TS-003-BLK-1.jpg … FAS-TS-003-BLK-5.jpg cover every Black size.</t>
   </si>
   <si>
-    <t>Free Size</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>12-15 Months</t>
+  </si>
+  <si>
+    <t>15-18 Months</t>
+  </si>
+  <si>
+    <t>18-21 Months</t>
+  </si>
+  <si>
+    <t>2-2.5 Years</t>
+  </si>
+  <si>
+    <t>2.5-3 Years</t>
+  </si>
+  <si>
+    <t>21-24 Months</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>2XL</t>
+  </si>
+  <si>
+    <t>3-3.5 Years</t>
+  </si>
+  <si>
+    <t>3.5-4 Years</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>3XL</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>4-4.5 Years</t>
+  </si>
+  <si>
+    <t>4.5-5 Years</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>4XL</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>5-5.5 Years</t>
+  </si>
+  <si>
+    <t>5.5-6 Years</t>
+  </si>
+  <si>
+    <t>5XL</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>6 Month</t>
+  </si>
+  <si>
+    <t>6-9 Months</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>8 Months</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>9-12 Months</t>
+  </si>
+  <si>
+    <t>Beetroot</t>
+  </si>
+  <si>
+    <t>Chocolate</t>
+  </si>
+  <si>
+    <t>Free size</t>
+  </si>
+  <si>
+    <t>IND-1</t>
+  </si>
+  <si>
+    <t>IND-10</t>
+  </si>
+  <si>
+    <t>IND-11</t>
+  </si>
+  <si>
+    <t>IND-12</t>
+  </si>
+  <si>
+    <t>IND-13</t>
+  </si>
+  <si>
+    <t>IND-2</t>
+  </si>
+  <si>
+    <t>IND-3</t>
+  </si>
+  <si>
+    <t>IND-4</t>
+  </si>
+  <si>
+    <t>IND-5</t>
+  </si>
+  <si>
+    <t>IND-6</t>
+  </si>
+  <si>
+    <t>IND-7</t>
+  </si>
+  <si>
+    <t>IND-8</t>
+  </si>
+  <si>
+    <t>IND-9</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Lemon</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>Mango</t>
+  </si>
+  <si>
+    <t>Rose</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>XL</t>
   </si>
   <si>
     <t>XS</t>
   </si>
   <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>XL</t>
-  </si>
-  <si>
     <t>XXL</t>
   </si>
   <si>
-    <t>3XL</t>
-  </si>
-  <si>
-    <t>4XL</t>
-  </si>
-  <si>
-    <t>5XL</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>IND-6</t>
-  </si>
-  <si>
-    <t>IND-7</t>
-  </si>
-  <si>
-    <t>IND-8</t>
-  </si>
-  <si>
-    <t>IND-9</t>
-  </si>
-  <si>
-    <t>IND-10</t>
+    <t>XXXL</t>
   </si>
   <si>
     <t>FAS-TS-003</t>
@@ -1253,7 +1394,7 @@
   <sheetPr>
     <tabColor rgb="FFF56C43"/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1391,548 +1532,590 @@
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+    <row r="19" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-    </row>
-    <row r="21" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+    </row>
+    <row r="22" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+    </row>
+    <row r="23" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
     </row>
     <row r="24" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
     </row>
-    <row r="25" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+    </row>
+    <row r="27" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+    </row>
+    <row r="28" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="29" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+    </row>
+    <row r="31" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+    </row>
+    <row r="32" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="30" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="16" t="s">
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B35" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B33" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B35" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="15" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="36" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B40" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C36" s="18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-    </row>
-    <row r="40" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B40" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C40" s="15" t="s">
-        <v>33</v>
+      <c r="C40" s="18" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="C41" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="16" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="42" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="19" t="s">
+      <c r="B42" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="C42" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C42" s="18" t="s">
+      <c r="B43" s="17" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="43" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="19" t="s">
+      <c r="C43" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="B43" s="17" t="s">
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C43" s="18" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="C44" s="18" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="45" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="B45" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" s="18" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="46" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="B46" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="C46" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="47" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B47" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="C47" s="18" t="s">
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+    </row>
+    <row r="47" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C47" s="15" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="48" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B50" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B51" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B52" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="C52" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="C48" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="49" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="20" t="s">
+    </row>
+    <row r="53" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B53" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="C49" s="18" t="s">
+      <c r="C53" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="16" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="50" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="20" t="s">
+      <c r="B54" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="B50" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="C50" s="18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-    </row>
-    <row r="54" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B54" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C54" s="15" t="s">
-        <v>33</v>
+      <c r="C54" s="18" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="55" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="16" t="s">
+      <c r="A56" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B56" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C56" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="C57" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B60" s="14"/>
+      <c r="C60" s="14"/>
+    </row>
+    <row r="61" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B61" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C56" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="57" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B57" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C57" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="58" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B58" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="C58" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="59" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B59" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C59" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="60" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B60" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C60" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="61" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B61" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C61" s="18" t="s">
+      <c r="C61" s="15" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="62" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B62" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C62" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B63" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C63" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B64" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C64" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B65" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C65" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="66" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B62" s="17" t="s">
+      <c r="B66" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C62" s="18" t="s">
+      <c r="C66" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="67" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="16" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="63" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B63" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="C63" s="18" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="64" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="B64" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="C64" s="18" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="65" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="B65" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="C65" s="18" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="66" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B66" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="C66" s="18" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="67" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" s="21" t="s">
-        <v>92</v>
-      </c>
       <c r="B67" s="17" t="s">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="C67" s="18" t="s">
-        <v>94</v>
+        <v>45</v>
       </c>
     </row>
     <row r="68" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="21" t="s">
-        <v>95</v>
+      <c r="A68" s="16" t="s">
+        <v>54</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="C68" s="18" t="s">
-        <v>97</v>
+        <v>45</v>
       </c>
     </row>
     <row r="69" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" s="22" t="s">
-        <v>98</v>
+      <c r="A69" s="16" t="s">
+        <v>56</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="C69" s="18" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
     </row>
     <row r="70" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="21" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="C70" s="18" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
     </row>
     <row r="71" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="21" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B71" s="17" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="C71" s="18" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
     </row>
     <row r="72" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="21" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="B72" s="17" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="C72" s="18" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
     </row>
     <row r="73" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="21" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="B73" s="17" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
     </row>
     <row r="74" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="21" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B74" s="17" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="C74" s="18" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
     </row>
     <row r="75" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="21" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="B75" s="17" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="C75" s="18" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
     </row>
     <row r="76" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" s="21" t="s">
-        <v>119</v>
+      <c r="A76" s="22" t="s">
+        <v>104</v>
       </c>
       <c r="B76" s="17" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="C76" s="18" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
     </row>
     <row r="77" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="B77" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="C77" s="18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="78" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="C78" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="79" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B79" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="C79" s="18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="80" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="B80" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C80" s="18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="81" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B81" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="C81" s="18" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="82" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B77" s="17" t="s">
+      <c r="B82" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="C77" s="18" t="s">
+      <c r="C82" s="18" t="s">
         <v>124</v>
       </c>
     </row>
+    <row r="83" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B83" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="C83" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="84" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="B84" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="C84" s="18" t="s">
+        <v>130</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="30">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A3:C3"/>
@@ -1949,14 +2132,20 @@
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A60:C60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1980,126 +2169,126 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D2" s="24">
         <v>1</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D3" s="25">
         <v>2</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B4" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" s="24" t="s">
         <v>137</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>131</v>
       </c>
       <c r="D4" s="24">
         <v>5</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D5" s="25">
         <v>3</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D7" s="25">
         <v>1</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
@@ -2108,7 +2297,7 @@
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -2117,7 +2306,7 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
@@ -2126,7 +2315,7 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -2135,7 +2324,7 @@
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
@@ -2157,7 +2346,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2165,117 +2354,322 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>178</v>
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -2301,39 +2695,39 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="28" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>180</v>
+        <v>227</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>181</v>
+        <v>228</v>
       </c>
       <c r="D2" s="28">
         <v>180</v>
@@ -2348,7 +2742,7 @@
         <v>3</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>182</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -2384,51 +2778,51 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B1" s="29" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E1" s="30" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="I1" s="30" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="J1" s="30" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="28" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>183</v>
+        <v>230</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>160</v>
+        <v>218</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>184</v>
+        <v>231</v>
       </c>
       <c r="E2" s="28" t="s">
-        <v>185</v>
+        <v>232</v>
       </c>
       <c r="F2" s="31">
         <v>499</v>
@@ -2440,27 +2834,27 @@
         <v>12</v>
       </c>
       <c r="I2" s="28" t="s">
-        <v>186</v>
+        <v>233</v>
       </c>
       <c r="J2" s="28" t="s">
-        <v>187</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="B3" s="33" t="s">
-        <v>183</v>
+        <v>230</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>161</v>
+        <v>216</v>
       </c>
       <c r="D3" s="33" t="s">
-        <v>188</v>
+        <v>235</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>185</v>
+        <v>232</v>
       </c>
       <c r="F3" s="34">
         <v>499</v>
@@ -2472,27 +2866,27 @@
         <v>18</v>
       </c>
       <c r="I3" s="33" t="s">
-        <v>186</v>
+        <v>233</v>
       </c>
       <c r="J3" s="33" t="s">
-        <v>187</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="28" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>189</v>
+        <v>236</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>160</v>
+        <v>218</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>190</v>
+        <v>237</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="F4" s="31">
         <v>499</v>
@@ -2504,27 +2898,27 @@
         <v>10</v>
       </c>
       <c r="I4" s="28" t="s">
-        <v>186</v>
+        <v>233</v>
       </c>
       <c r="J4" s="28" t="s">
-        <v>187</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>189</v>
+        <v>236</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>161</v>
+        <v>216</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>191</v>
+        <v>238</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="F5" s="34">
         <v>499</v>
@@ -2536,17 +2930,17 @@
         <v>8</v>
       </c>
       <c r="I5" s="33" t="s">
-        <v>186</v>
+        <v>233</v>
       </c>
       <c r="J5" s="33" t="s">
-        <v>187</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Size" prompt="Pick one size from the list." showErrorMessage="1" errorTitle="Size" error="Pick a size from the Size dropdown (admin Size attributes)." sqref="C2:C200">
-      <formula1>'Size Names'!$A$2:$A$23</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Size" prompt="Pick a size from the list, or type several for this colour as 6,7,8,9. Kids Fashion: choose an age-group size (6-9 Months, 2-2.5 Years)." errorTitle="Size" error="Pick one size from the Size dropdown (admin Size attributes)." sqref="C2:C200">
+      <formula1>'Size Names'!$A$2:$A$64</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Status" prompt="out_of_stock rows are skipped on submit." showErrorMessage="1" errorTitle="Status" error="Pick one of: in_stock, out_of_stock" sqref="J2:J200">
       <formula1>"in_stock,out_of_stock"</formula1>
@@ -2587,84 +2981,84 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="O1" s="37" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="T1" s="36" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="V1" s="36" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="28" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>180</v>
+        <v>227</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>181</v>
+        <v>228</v>
       </c>
       <c r="D2" s="28">
         <v>180</v>
@@ -2679,52 +3073,52 @@
         <v>3</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>182</v>
+        <v>229</v>
       </c>
       <c r="I2" s="28" t="s">
-        <v>192</v>
+        <v>239</v>
       </c>
       <c r="J2" s="28" t="s">
-        <v>193</v>
+        <v>240</v>
       </c>
       <c r="K2" s="28" t="s">
-        <v>194</v>
+        <v>241</v>
       </c>
       <c r="L2" s="28" t="s">
-        <v>195</v>
+        <v>242</v>
       </c>
       <c r="M2" s="28" t="s">
-        <v>196</v>
+        <v>243</v>
       </c>
       <c r="N2" s="32">
         <v>5</v>
       </c>
       <c r="O2" s="28" t="s">
-        <v>197</v>
+        <v>244</v>
       </c>
       <c r="P2" s="38" t="s">
-        <v>198</v>
+        <v>245</v>
       </c>
       <c r="Q2" s="38" t="s">
-        <v>199</v>
+        <v>246</v>
       </c>
       <c r="R2" s="38" t="s">
-        <v>200</v>
+        <v>247</v>
       </c>
       <c r="S2" s="38" t="s">
-        <v>201</v>
+        <v>248</v>
       </c>
       <c r="T2" s="38" t="s">
-        <v>202</v>
+        <v>249</v>
       </c>
       <c r="U2" s="28" t="s">
-        <v>203</v>
+        <v>250</v>
       </c>
       <c r="V2" s="38" t="s">
-        <v>204</v>
+        <v>251</v>
       </c>
       <c r="W2" s="28" t="s">
-        <v>205</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>